<commit_message>
Actualizar interfaz web con boton Administrador destacado
</commit_message>
<xml_diff>
--- a/Precios_Metales_COP.xlsx
+++ b/Precios_Metales_COP.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Dashboard y Gráficos" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Precios Diarios" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard y Gráficos" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Precios Diarios" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Precios Diarios'!$A$1:$H$463</definedName>
@@ -273,14 +273,14 @@
 </file>
 
 <file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <style val="13"/>
   <chart>
     <title>
       <tx>
         <rich>
-          <a:bodyPr/>
-          <a:p>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
             <a:pPr>
               <a:defRPr/>
             </a:pPr>
@@ -303,7 +303,7 @@
             </strRef>
           </tx>
           <spPr>
-            <a:ln w="22000">
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="22000">
               <a:solidFill>
                 <a:srgbClr val="D97706"/>
               </a:solidFill>
@@ -314,7 +314,7 @@
             <symbol val="circle"/>
             <size val="3"/>
             <spPr>
-              <a:ln>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:prstDash val="solid"/>
               </a:ln>
             </spPr>
@@ -343,8 +343,8 @@
         <title>
           <tx>
             <rich>
-              <a:bodyPr/>
-              <a:p>
+              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:pPr>
                   <a:defRPr/>
                 </a:pPr>
@@ -372,8 +372,8 @@
         <title>
           <tx>
             <rich>
-              <a:bodyPr/>
-              <a:p>
+              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:pPr>
                   <a:defRPr/>
                 </a:pPr>
@@ -398,14 +398,14 @@
 </file>
 
 <file path=xl/charts/chart2.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <style val="13"/>
   <chart>
     <title>
       <tx>
         <rich>
-          <a:bodyPr/>
-          <a:p>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
             <a:pPr>
               <a:defRPr/>
             </a:pPr>
@@ -428,7 +428,7 @@
             </strRef>
           </tx>
           <spPr>
-            <a:ln w="22000">
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="22000">
               <a:solidFill>
                 <a:srgbClr val="475569"/>
               </a:solidFill>
@@ -439,7 +439,7 @@
             <symbol val="circle"/>
             <size val="3"/>
             <spPr>
-              <a:ln>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:prstDash val="solid"/>
               </a:ln>
             </spPr>
@@ -468,8 +468,8 @@
         <title>
           <tx>
             <rich>
-              <a:bodyPr/>
-              <a:p>
+              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:pPr>
                   <a:defRPr/>
                 </a:pPr>
@@ -497,8 +497,8 @@
         <title>
           <tx>
             <rich>
-              <a:bodyPr/>
-              <a:p>
+              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:pPr>
                   <a:defRPr/>
                 </a:pPr>
@@ -523,14 +523,14 @@
 </file>
 
 <file path=xl/charts/chart3.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <style val="13"/>
   <chart>
     <title>
       <tx>
         <rich>
-          <a:bodyPr/>
-          <a:p>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
             <a:pPr>
               <a:defRPr/>
             </a:pPr>
@@ -553,7 +553,7 @@
             </strRef>
           </tx>
           <spPr>
-            <a:ln>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:solidFill>
                 <a:srgbClr val="D97706"/>
               </a:solidFill>
@@ -563,7 +563,7 @@
           <marker>
             <symbol val="none"/>
             <spPr>
-              <a:ln>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:prstDash val="solid"/>
               </a:ln>
             </spPr>
@@ -593,7 +593,7 @@
             </strRef>
           </tx>
           <spPr>
-            <a:ln>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:solidFill>
                 <a:srgbClr val="475569"/>
               </a:solidFill>
@@ -603,7 +603,7 @@
           <marker>
             <symbol val="none"/>
             <spPr>
-              <a:ln>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:prstDash val="solid"/>
               </a:ln>
             </spPr>
@@ -627,8 +627,8 @@
         <title>
           <tx>
             <rich>
-              <a:bodyPr/>
-              <a:p>
+              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:pPr>
                   <a:defRPr/>
                 </a:pPr>
@@ -656,8 +656,8 @@
         <title>
           <tx>
             <rich>
-              <a:bodyPr/>
-              <a:p>
+              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:pPr>
                   <a:defRPr/>
                 </a:pPr>
@@ -685,8 +685,8 @@
         <title>
           <tx>
             <rich>
-              <a:bodyPr/>
-              <a:p>
+              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:pPr>
                   <a:defRPr/>
                 </a:pPr>
@@ -715,7 +715,7 @@
 </file>
 
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
-<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <oneCellAnchor>
     <from>
       <col>0</col>
@@ -730,9 +730,9 @@
         <cNvGraphicFramePr/>
       </nvGraphicFramePr>
       <xfrm/>
-      <a:graphic>
+      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart r:id="rId1"/>
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
@@ -752,9 +752,9 @@
         <cNvGraphicFramePr/>
       </nvGraphicFramePr>
       <xfrm/>
-      <a:graphic>
+      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart r:id="rId2"/>
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId2"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
@@ -774,9 +774,9 @@
         <cNvGraphicFramePr/>
       </nvGraphicFramePr>
       <xfrm/>
-      <a:graphic>
+      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart r:id="rId3"/>
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId3"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
@@ -21616,13 +21616,13 @@
         <v>46245</v>
       </c>
       <c r="B463" s="19" t="n">
-        <v>4431.7998046875</v>
+        <v>4428.2001953125</v>
       </c>
       <c r="C463" s="19" t="n">
-        <v>64.97499847412109</v>
+        <v>64.83999633789062</v>
       </c>
       <c r="D463" s="19" t="n">
-        <v>3127.47998046875</v>
+        <v>3128.949951171875</v>
       </c>
       <c r="E463" s="20">
         <f>ROUND((B463/31.1034768)*D463, 2)</f>

</xml_diff>

<commit_message>
🤖 Actualización automática diaria [GitHub Actions]
</commit_message>
<xml_diff>
--- a/Precios_Metales_COP.xlsx
+++ b/Precios_Metales_COP.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard y Gráficos" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Precios Diarios" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Dashboard y Gráficos" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Precios Diarios" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Precios Diarios'!$A$1:$H$463</definedName>
@@ -273,14 +273,14 @@
 </file>
 
 <file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <style val="13"/>
   <chart>
     <title>
       <tx>
         <rich>
-          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:bodyPr/>
+          <a:p>
             <a:pPr>
               <a:defRPr/>
             </a:pPr>
@@ -303,7 +303,7 @@
             </strRef>
           </tx>
           <spPr>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="22000">
+            <a:ln w="22000">
               <a:solidFill>
                 <a:srgbClr val="D97706"/>
               </a:solidFill>
@@ -314,7 +314,7 @@
             <symbol val="circle"/>
             <size val="3"/>
             <spPr>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:ln>
                 <a:prstDash val="solid"/>
               </a:ln>
             </spPr>
@@ -343,8 +343,8 @@
         <title>
           <tx>
             <rich>
-              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:bodyPr/>
+              <a:p>
                 <a:pPr>
                   <a:defRPr/>
                 </a:pPr>
@@ -372,8 +372,8 @@
         <title>
           <tx>
             <rich>
-              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:bodyPr/>
+              <a:p>
                 <a:pPr>
                   <a:defRPr/>
                 </a:pPr>
@@ -398,14 +398,14 @@
 </file>
 
 <file path=xl/charts/chart2.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <style val="13"/>
   <chart>
     <title>
       <tx>
         <rich>
-          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:bodyPr/>
+          <a:p>
             <a:pPr>
               <a:defRPr/>
             </a:pPr>
@@ -428,7 +428,7 @@
             </strRef>
           </tx>
           <spPr>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="22000">
+            <a:ln w="22000">
               <a:solidFill>
                 <a:srgbClr val="475569"/>
               </a:solidFill>
@@ -439,7 +439,7 @@
             <symbol val="circle"/>
             <size val="3"/>
             <spPr>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:ln>
                 <a:prstDash val="solid"/>
               </a:ln>
             </spPr>
@@ -468,8 +468,8 @@
         <title>
           <tx>
             <rich>
-              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:bodyPr/>
+              <a:p>
                 <a:pPr>
                   <a:defRPr/>
                 </a:pPr>
@@ -497,8 +497,8 @@
         <title>
           <tx>
             <rich>
-              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:bodyPr/>
+              <a:p>
                 <a:pPr>
                   <a:defRPr/>
                 </a:pPr>
@@ -523,14 +523,14 @@
 </file>
 
 <file path=xl/charts/chart3.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <style val="13"/>
   <chart>
     <title>
       <tx>
         <rich>
-          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:bodyPr/>
+          <a:p>
             <a:pPr>
               <a:defRPr/>
             </a:pPr>
@@ -553,7 +553,7 @@
             </strRef>
           </tx>
           <spPr>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:ln>
               <a:solidFill>
                 <a:srgbClr val="D97706"/>
               </a:solidFill>
@@ -563,7 +563,7 @@
           <marker>
             <symbol val="none"/>
             <spPr>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:ln>
                 <a:prstDash val="solid"/>
               </a:ln>
             </spPr>
@@ -593,7 +593,7 @@
             </strRef>
           </tx>
           <spPr>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:ln>
               <a:solidFill>
                 <a:srgbClr val="475569"/>
               </a:solidFill>
@@ -603,7 +603,7 @@
           <marker>
             <symbol val="none"/>
             <spPr>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:ln>
                 <a:prstDash val="solid"/>
               </a:ln>
             </spPr>
@@ -627,8 +627,8 @@
         <title>
           <tx>
             <rich>
-              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:bodyPr/>
+              <a:p>
                 <a:pPr>
                   <a:defRPr/>
                 </a:pPr>
@@ -656,8 +656,8 @@
         <title>
           <tx>
             <rich>
-              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:bodyPr/>
+              <a:p>
                 <a:pPr>
                   <a:defRPr/>
                 </a:pPr>
@@ -685,8 +685,8 @@
         <title>
           <tx>
             <rich>
-              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:bodyPr/>
+              <a:p>
                 <a:pPr>
                   <a:defRPr/>
                 </a:pPr>
@@ -715,7 +715,7 @@
 </file>
 
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
-<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <oneCellAnchor>
     <from>
       <col>0</col>
@@ -730,9 +730,9 @@
         <cNvGraphicFramePr/>
       </nvGraphicFramePr>
       <xfrm/>
-      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+      <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+          <c:chart r:id="rId1"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
@@ -752,9 +752,9 @@
         <cNvGraphicFramePr/>
       </nvGraphicFramePr>
       <xfrm/>
-      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+      <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId2"/>
+          <c:chart r:id="rId2"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
@@ -774,9 +774,9 @@
         <cNvGraphicFramePr/>
       </nvGraphicFramePr>
       <xfrm/>
-      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+      <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId3"/>
+          <c:chart r:id="rId3"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
@@ -21619,10 +21619,10 @@
         <v>4428.2001953125</v>
       </c>
       <c r="C463" s="19" t="n">
-        <v>64.83999633789062</v>
+        <v>64.80500030517578</v>
       </c>
       <c r="D463" s="19" t="n">
-        <v>3128.949951171875</v>
+        <v>3128.97998046875</v>
       </c>
       <c r="E463" s="20">
         <f>ROUND((B463/31.1034768)*D463, 2)</f>

</xml_diff>

<commit_message>
Actualizar READMEs con enlaces de acceso rapido y guia para celular
</commit_message>
<xml_diff>
--- a/Precios_Metales_COP.xlsx
+++ b/Precios_Metales_COP.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Dashboard y Gráficos" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Precios Diarios" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard y Gráficos" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Precios Diarios" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Precios Diarios'!$A$1:$H$463</definedName>
@@ -273,14 +273,14 @@
 </file>
 
 <file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <style val="13"/>
   <chart>
     <title>
       <tx>
         <rich>
-          <a:bodyPr/>
-          <a:p>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
             <a:pPr>
               <a:defRPr/>
             </a:pPr>
@@ -303,7 +303,7 @@
             </strRef>
           </tx>
           <spPr>
-            <a:ln w="22000">
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="22000">
               <a:solidFill>
                 <a:srgbClr val="D97706"/>
               </a:solidFill>
@@ -314,7 +314,7 @@
             <symbol val="circle"/>
             <size val="3"/>
             <spPr>
-              <a:ln>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:prstDash val="solid"/>
               </a:ln>
             </spPr>
@@ -343,8 +343,8 @@
         <title>
           <tx>
             <rich>
-              <a:bodyPr/>
-              <a:p>
+              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:pPr>
                   <a:defRPr/>
                 </a:pPr>
@@ -372,8 +372,8 @@
         <title>
           <tx>
             <rich>
-              <a:bodyPr/>
-              <a:p>
+              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:pPr>
                   <a:defRPr/>
                 </a:pPr>
@@ -398,14 +398,14 @@
 </file>
 
 <file path=xl/charts/chart2.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <style val="13"/>
   <chart>
     <title>
       <tx>
         <rich>
-          <a:bodyPr/>
-          <a:p>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
             <a:pPr>
               <a:defRPr/>
             </a:pPr>
@@ -428,7 +428,7 @@
             </strRef>
           </tx>
           <spPr>
-            <a:ln w="22000">
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="22000">
               <a:solidFill>
                 <a:srgbClr val="475569"/>
               </a:solidFill>
@@ -439,7 +439,7 @@
             <symbol val="circle"/>
             <size val="3"/>
             <spPr>
-              <a:ln>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:prstDash val="solid"/>
               </a:ln>
             </spPr>
@@ -468,8 +468,8 @@
         <title>
           <tx>
             <rich>
-              <a:bodyPr/>
-              <a:p>
+              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:pPr>
                   <a:defRPr/>
                 </a:pPr>
@@ -497,8 +497,8 @@
         <title>
           <tx>
             <rich>
-              <a:bodyPr/>
-              <a:p>
+              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:pPr>
                   <a:defRPr/>
                 </a:pPr>
@@ -523,14 +523,14 @@
 </file>
 
 <file path=xl/charts/chart3.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <style val="13"/>
   <chart>
     <title>
       <tx>
         <rich>
-          <a:bodyPr/>
-          <a:p>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
             <a:pPr>
               <a:defRPr/>
             </a:pPr>
@@ -553,7 +553,7 @@
             </strRef>
           </tx>
           <spPr>
-            <a:ln>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:solidFill>
                 <a:srgbClr val="D97706"/>
               </a:solidFill>
@@ -563,7 +563,7 @@
           <marker>
             <symbol val="none"/>
             <spPr>
-              <a:ln>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:prstDash val="solid"/>
               </a:ln>
             </spPr>
@@ -593,7 +593,7 @@
             </strRef>
           </tx>
           <spPr>
-            <a:ln>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:solidFill>
                 <a:srgbClr val="475569"/>
               </a:solidFill>
@@ -603,7 +603,7 @@
           <marker>
             <symbol val="none"/>
             <spPr>
-              <a:ln>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:prstDash val="solid"/>
               </a:ln>
             </spPr>
@@ -627,8 +627,8 @@
         <title>
           <tx>
             <rich>
-              <a:bodyPr/>
-              <a:p>
+              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:pPr>
                   <a:defRPr/>
                 </a:pPr>
@@ -656,8 +656,8 @@
         <title>
           <tx>
             <rich>
-              <a:bodyPr/>
-              <a:p>
+              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:pPr>
                   <a:defRPr/>
                 </a:pPr>
@@ -685,8 +685,8 @@
         <title>
           <tx>
             <rich>
-              <a:bodyPr/>
-              <a:p>
+              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:pPr>
                   <a:defRPr/>
                 </a:pPr>
@@ -715,7 +715,7 @@
 </file>
 
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
-<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <oneCellAnchor>
     <from>
       <col>0</col>
@@ -730,9 +730,9 @@
         <cNvGraphicFramePr/>
       </nvGraphicFramePr>
       <xfrm/>
-      <a:graphic>
+      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart r:id="rId1"/>
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
@@ -752,9 +752,9 @@
         <cNvGraphicFramePr/>
       </nvGraphicFramePr>
       <xfrm/>
-      <a:graphic>
+      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart r:id="rId2"/>
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId2"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
@@ -774,9 +774,9 @@
         <cNvGraphicFramePr/>
       </nvGraphicFramePr>
       <xfrm/>
-      <a:graphic>
+      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart r:id="rId3"/>
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId3"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
@@ -21616,10 +21616,10 @@
         <v>46245</v>
       </c>
       <c r="B463" s="19" t="n">
-        <v>4428.2001953125</v>
+        <v>4427.2001953125</v>
       </c>
       <c r="C463" s="19" t="n">
-        <v>64.80500030517578</v>
+        <v>64.80999755859375</v>
       </c>
       <c r="D463" s="19" t="n">
         <v>3128.97998046875</v>

</xml_diff>